<commit_message>
Modify the Excel files to reflect the changes by adding the --auto and --script test cases
</commit_message>
<xml_diff>
--- a/docs/test_case.xlsx
+++ b/docs/test_case.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cpp-fsoft\parking_cplus-main\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73D9253F-7AE2-40EC-AFEE-597D1C28E69E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89F7E5EE-5AD6-4E58-8E97-37E1C9880A92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="2250" windowWidth="20595" windowHeight="11970" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8175" yWindow="1725" windowWidth="20595" windowHeight="11970" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Report" sheetId="1" r:id="rId1"/>
@@ -20,291 +20,321 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="105">
+  <si>
+    <t>Loại</t>
+  </si>
   <si>
     <t>ID</t>
   </si>
   <si>
+    <t>Trường hợp</t>
+  </si>
+  <si>
+    <t>Đầu vào hoặc thao tác</t>
+  </si>
+  <si>
+    <t>Kết quả mong đợi</t>
+  </si>
+  <si>
+    <t>Kết quả thực tế</t>
+  </si>
+  <si>
+    <t>Trạng thái</t>
+  </si>
+  <si>
     <t>Normal</t>
   </si>
   <si>
     <t>TC-NORM-01</t>
   </si>
   <si>
+    <t>Biển số xe 4 số cuối</t>
+  </si>
+  <si>
+    <t>Chọn 1, ID: 18A-0298</t>
+  </si>
+  <si>
+    <t>Mở barrier vào, gán vị trí P1</t>
+  </si>
+  <si>
+    <t>Như mong đợi</t>
+  </si>
+  <si>
+    <t>ĐẠT</t>
+  </si>
+  <si>
     <t>TC-NORM-02</t>
   </si>
   <si>
+    <t>Biển số xe 5 số cuối, đã có xe ở P1</t>
+  </si>
+  <si>
+    <t>Chọn 1, ID: 28D-19213</t>
+  </si>
+  <si>
+    <t>Mở barrier vào, gán vị trí còn trống tiếp theo (P2)</t>
+  </si>
+  <si>
     <t>TC-NORM-03</t>
   </si>
   <si>
+    <t>Biển số xe 5 số cuối có dấu . hợp lệ</t>
+  </si>
+  <si>
+    <t>Chọn 1, ID: 30A-123.45 / 88E-929.10</t>
+  </si>
+  <si>
+    <t>Mở barrier vào, gán vị trí</t>
+  </si>
+  <si>
     <t>TC-NORM-04</t>
   </si>
   <si>
+    <t>Xe trong bãi xe đi ra</t>
+  </si>
+  <si>
+    <t>Chọn 2, ID: 18A-0298 (đã gán vị trí P1 tại TC-NORM-01)</t>
+  </si>
+  <si>
+    <t>Mở barrier ra, giải phóng vị trí P1</t>
+  </si>
+  <si>
     <t>TC-NORM-05</t>
   </si>
   <si>
+    <t>Kiểm tra trạng thái</t>
+  </si>
+  <si>
+    <t>Chọn 3</t>
+  </si>
+  <si>
+    <t>Xem bản đồ đỗ xe và lịch sử các xe đang đỗ</t>
+  </si>
+  <si>
     <t>TC-NORM-06</t>
   </si>
   <si>
+    <t>Thoát hệ thống thông thường</t>
+  </si>
+  <si>
+    <t>Chọn 0</t>
+  </si>
+  <si>
+    <t>Thoát ra an toàn (mã thoát 0)</t>
+  </si>
+  <si>
     <t>TC-NORM-07</t>
   </si>
   <si>
+    <t>Phân lại slot để xe</t>
+  </si>
+  <si>
+    <t>Chọn 2, nhập ID xe ở slot P1, sau đó chọn 1 và nhập ID xe mới vào</t>
+  </si>
+  <si>
+    <t>Slot P1 vừa giải phóng được tái sử dụng</t>
+  </si>
+  <si>
     <t>TC-NORM-08</t>
   </si>
   <si>
+    <t>Tự động đưa xe từ hàng đợi vào</t>
+  </si>
+  <si>
+    <t>Lấp đầy hết chỗ trong bãi, chọn 1 và nhập ID xe cần vào, sau đó chọn 2 và nhập ID xe trong bãi cần ra</t>
+  </si>
+  <si>
+    <t>Vị trí được giải phóng sẽ tự động được gán cho xe đầu tiên trong hàng đợi</t>
+  </si>
+  <si>
     <t>Boundary</t>
   </si>
   <si>
     <t>TC-BOUND-01</t>
   </si>
   <si>
+    <t>Biển số xe độ dài hợp lệ ngắn nhất</t>
+  </si>
+  <si>
+    <t>Chấp nhận biển số xe hợp lệ</t>
+  </si>
+  <si>
     <t>TC-BOUND-02</t>
   </si>
   <si>
+    <t>Biển số xe độ dài hợp lệ dài nhất</t>
+  </si>
+  <si>
+    <t>Chọn 1, ID: 30A-123.45</t>
+  </si>
+  <si>
     <t>TC-BOUND-03</t>
   </si>
   <si>
+    <t>Hàng đợi khi bãi xe đầy</t>
+  </si>
+  <si>
+    <t>Lấp đầy bãi xe. Chọn 1, ID: 99A-888.88</t>
+  </si>
+  <si>
+    <t>Đặt trong hàng đợi, barrier vào vẫn đóng</t>
+  </si>
+  <si>
     <t>TC-BOUND-04</t>
   </si>
   <si>
+    <t>Xe vừa vào đã ra</t>
+  </si>
+  <si>
+    <t>Chọn 1, nhập ID xe, sau đó chọn 2 và nhập cùng ID xe đó</t>
+  </si>
+  <si>
+    <t>Thao tác được chấp nhận</t>
+  </si>
+  <si>
     <t>Abnormal</t>
   </si>
   <si>
     <t>TC-ABNORM-01</t>
   </si>
   <si>
+    <t>Từ chối biển số xe không hợp lệ</t>
+  </si>
+  <si>
+    <t>Chọn 1, rồi nhập ID bất kỳ: F27839 / !93J918@ / MS-029 / 11X-222 / 39Y-144785 / 30N 7812</t>
+  </si>
+  <si>
+    <t>Báo từ chối do biển số xe không hợp lệ</t>
+  </si>
+  <si>
     <t>TC-ABNORM-02</t>
   </si>
   <si>
+    <t>Từ chối biển số xe máy</t>
+  </si>
+  <si>
+    <t>Chọn 1, ID: 29LD-29180</t>
+  </si>
+  <si>
+    <t>Báo từ chối do biển số xe không hợp lệ (chỉ chấp nhận ô tô)</t>
+  </si>
+  <si>
     <t>TC-ABNORM-03</t>
   </si>
   <si>
+    <t>Đầu vào là chữ</t>
+  </si>
+  <si>
+    <t>Chọn: xyz</t>
+  </si>
+  <si>
+    <t>Báo lỗi lựa chọn không hợp lệ</t>
+  </si>
+  <si>
     <t>TC-ABNORM-04</t>
   </si>
   <si>
+    <t>Đầu vào trống hoặc không đúng lựa chọn</t>
+  </si>
+  <si>
+    <t>Chọn: bấm Enter hoặc chọn 4, 5, 6…</t>
+  </si>
+  <si>
     <t>TC-ABNORM-05</t>
   </si>
   <si>
+    <t>Xe cần vào có ID trùng với xe đã đỗ</t>
+  </si>
+  <si>
+    <t>Chọn 1 và nhập ID 18A-0298 khi xe còn trong bãi</t>
+  </si>
+  <si>
+    <t>Báo từ chối do trùng với xe đang có trong bãi</t>
+  </si>
+  <si>
     <t>TC-ABNORM-06</t>
   </si>
   <si>
+    <t>Xe cần ra không có trong bãi</t>
+  </si>
+  <si>
+    <t>Chọn 2 và nhập ID không có trong bãi: 99A-999.99</t>
+  </si>
+  <si>
+    <t>Báo từ chối do không có xe đó trong bãi</t>
+  </si>
+  <si>
+    <t>TC-ABNORM-08</t>
+  </si>
+  <si>
+    <t>Thiếu thư mục logs hoặc file system.log</t>
+  </si>
+  <si>
+    <t>Xóa thư mục logs hoặc file system.log trong thư mục đó và khởi động app</t>
+  </si>
+  <si>
+    <t>File system.log được tạo tự động ngay khi khởi động</t>
+  </si>
+  <si>
+    <t>Note:</t>
+  </si>
+  <si>
+    <t>Trường hợp bình thường</t>
+  </si>
+  <si>
+    <t>Trường hợp biên</t>
+  </si>
+  <si>
+    <t>Trường hợp bất thường</t>
+  </si>
+  <si>
+    <t>TC-NORM-09</t>
+  </si>
+  <si>
+    <t>Chạy chế độ tự động (--auto)</t>
+  </si>
+  <si>
+    <t>Sinh 10 sự kiện vào/ra ngẫu nhiên, tự động điều phối barrier và kết thúc an toàn</t>
+  </si>
+  <si>
+    <t>TC-NORM-10</t>
+  </si>
+  <si>
+    <t>Chạy kịch bản từ file script (--script)</t>
+  </si>
+  <si>
+    <t>Đọc và thực thi từng lệnh trong file script (ENTRY, WAIT, STATUS, EXIT, QUIT) thành công</t>
+  </si>
+  <si>
     <t>TC-ABNORM-07</t>
   </si>
   <si>
-    <t>TC-ABNORM-08</t>
-  </si>
-  <si>
-    <t>Loại</t>
-  </si>
-  <si>
-    <t>Trường hợp</t>
-  </si>
-  <si>
-    <t>Đầu vào hoặc thao tác</t>
-  </si>
-  <si>
-    <t>Kết quả mong đợi</t>
-  </si>
-  <si>
-    <t>Kết quả thực tế</t>
-  </si>
-  <si>
-    <t>Trạng thái</t>
-  </si>
-  <si>
-    <t>Note:</t>
-  </si>
-  <si>
-    <t>Trường hợp bình thường</t>
-  </si>
-  <si>
-    <t>Trường hợp biên</t>
-  </si>
-  <si>
-    <t>Trường hợp bất thường</t>
-  </si>
-  <si>
-    <t>Biển số xe 4 số cuối</t>
-  </si>
-  <si>
-    <t>Chọn 1, ID: 18A-0298</t>
-  </si>
-  <si>
-    <t>Chọn 1, ID: 28D-19213</t>
-  </si>
-  <si>
-    <t>Chọn 1, ID: 30A-123.45 / 88E-929.10</t>
-  </si>
-  <si>
-    <t>Chọn 3</t>
-  </si>
-  <si>
-    <t>Chọn 0</t>
-  </si>
-  <si>
-    <t>Chọn 1, ID: 30A-123.45</t>
-  </si>
-  <si>
-    <t>Chọn 1, ID: 29LD-29180</t>
-  </si>
-  <si>
-    <t>Mở barrier vào, gán vị trí P1</t>
-  </si>
-  <si>
-    <t>Như mong đợi</t>
-  </si>
-  <si>
-    <t>ĐẠT</t>
-  </si>
-  <si>
-    <t>Mở barrier vào, gán vị trí còn trống tiếp theo (P2)</t>
-  </si>
-  <si>
-    <t>Biển số xe 5 số cuối, đã có xe ở P1</t>
-  </si>
-  <si>
-    <t>Biển số xe 5 số cuối có dấu . hợp lệ</t>
-  </si>
-  <si>
-    <t>Mở barrier vào, gán vị trí</t>
-  </si>
-  <si>
-    <t>Xe trong bãi xe đi ra</t>
-  </si>
-  <si>
-    <t>Mở barrier ra, giải phóng vị trí P1</t>
-  </si>
-  <si>
-    <t>Chọn 2, ID: 18A-0298 (đã gán vị trí P1 tại TC-NORM-01)</t>
-  </si>
-  <si>
-    <t>Kiểm tra trạng thái</t>
-  </si>
-  <si>
-    <t>Xem bản đồ đỗ xe và lịch sử các xe đang đỗ</t>
-  </si>
-  <si>
-    <t>Thoát hệ thống thông thường</t>
-  </si>
-  <si>
-    <t>Thoát ra an toàn (mã thoát 0)</t>
-  </si>
-  <si>
-    <t>Phân lại slot để xe</t>
-  </si>
-  <si>
-    <t>Chọn 2, nhập ID xe ở slot P1, sau đó chọn 1 và nhập ID xe mới vào</t>
-  </si>
-  <si>
-    <t>Slot P1 vừa giải phóng được tái sử dụng</t>
-  </si>
-  <si>
-    <t>Tự động đưa xe từ hàng đợi vào</t>
-  </si>
-  <si>
-    <t>Lấp đầy hết chỗ trong bãi, chọn 1 và nhập ID xe cần vào, sau đó chọn 2 và nhập ID xe trong bãi cần ra</t>
-  </si>
-  <si>
-    <t>Vị trí được giải phóng sẽ tự động được gán cho xe đầu tiên trong hàng đợi</t>
-  </si>
-  <si>
-    <t>Biển số xe độ dài hợp lệ ngắn nhất</t>
-  </si>
-  <si>
-    <t>Biển số xe độ dài hợp lệ dài nhất</t>
-  </si>
-  <si>
-    <t>Chấp nhận biển số xe hợp lệ</t>
-  </si>
-  <si>
-    <t>Hàng đợi khi bãi xe đầy</t>
-  </si>
-  <si>
-    <t>Lấp đầy bãi xe. Chọn 1, ID: 99A-888.88</t>
-  </si>
-  <si>
-    <t>Đặt trong hàng đợi, barrier vào vẫn đóng</t>
-  </si>
-  <si>
-    <t>Xe vừa vào đã ra</t>
-  </si>
-  <si>
-    <t>Chọn 1, nhập ID xe, sau đó chọn 2 và nhập cùng ID xe đó</t>
-  </si>
-  <si>
-    <t>Thao tác được chấp nhận</t>
-  </si>
-  <si>
-    <t>Từ chối biển số xe không hợp lệ</t>
-  </si>
-  <si>
-    <t>Chọn 1, rồi nhập ID bất kỳ: F27839 / !93J918@ / MS-029 / 11X-222 / 39Y-144785 / 30N 7812</t>
-  </si>
-  <si>
-    <t>Báo từ chối do biển số xe không hợp lệ</t>
-  </si>
-  <si>
-    <t>Từ chối biển số xe máy</t>
-  </si>
-  <si>
-    <t>Báo từ chối do biển số xe không hợp lệ (chỉ chấp nhận ô tô)</t>
-  </si>
-  <si>
-    <t>Đầu vào là chữ</t>
-  </si>
-  <si>
-    <t>Chọn: xyz</t>
-  </si>
-  <si>
-    <t>Báo lỗi lựa chọn không hợp lệ</t>
-  </si>
-  <si>
-    <t>Đầu vào trống hoặc không đúng lựa chọn</t>
-  </si>
-  <si>
-    <t>Chọn: bấm Enter hoặc chọn 4, 5, 6…</t>
-  </si>
-  <si>
-    <t>Chọn 1 và nhập ID 18A-0298 khi xe còn trong bãi</t>
-  </si>
-  <si>
-    <t>Báo từ chối do trùng với xe đang có trong bãi</t>
-  </si>
-  <si>
-    <t>Xe cần vào có ID trùng với xe đã đỗ</t>
-  </si>
-  <si>
-    <t>Xe cần ra không có trong bãi</t>
-  </si>
-  <si>
-    <t>Chọn 2 và nhập ID không có trong bãi: 99A-999.99</t>
-  </si>
-  <si>
-    <t>Báo từ chối do không có xe đó trong bãi</t>
-  </si>
-  <si>
-    <t>Lấp đầy bãi xe. Chọn 1 rồi nhập ID 99A-888.88, lặp lại 2 lần</t>
-  </si>
-  <si>
-    <t>Báo từ chối do xe đang có trong hàng đợi</t>
-  </si>
-  <si>
-    <t>Hàng đợi nhận 2 xe cùng ID</t>
-  </si>
-  <si>
-    <t>KHÔNG ĐẠT</t>
-  </si>
-  <si>
-    <t>ID xe cần vào trùng với xe khác trong hàng đợi</t>
-  </si>
-  <si>
-    <t>Thiếu thư mục logs hoặc file system.log</t>
-  </si>
-  <si>
-    <t>Xóa thư mục logs hoặc file system.log trong thư mục đó và khởi động app</t>
-  </si>
-  <si>
-    <t>File system.log được tạo tự động ngay khi khởi động</t>
+    <t>Kết hợp tham số --auto và --script đồng thời</t>
+  </si>
+  <si>
+    <t>Báo lỗi không cho phép kết hợp 2 tham số, trả mã thoát 1 và dừng</t>
+  </si>
+  <si>
+    <t>Đường dẫn file script không tồn tại</t>
+  </si>
+  <si>
+    <t>Báo lỗi không mở được file script, trả mã thoát 1 và dừng</t>
+  </si>
+  <si>
+    <t>TC-ABNORM-09</t>
+  </si>
+  <si>
+    <t>Chạy câu lệnh .\smart_parking.exe --auto 10 --interval 500</t>
+  </si>
+  <si>
+    <t>Chạy câu lệnh .\smart_parking.exe --script scripts/demo.txt --interval 500</t>
+  </si>
+  <si>
+    <t>Chạy câu lệnh .\smart_parking.exe --auto 5 --script scripts/demo.txt</t>
+  </si>
+  <si>
+    <t>Chạy câu lệnh .\smart_parking.exe --script scripts/not_found.txt</t>
   </si>
 </sst>
 </file>
@@ -360,16 +390,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F8013BFF-45F9-4366-81C7-84EB6D6C169B}" name="Table1" displayName="Table1" ref="A1:G21" totalsRowShown="0">
-  <autoFilter ref="A1:G21" xr:uid="{F8013BFF-45F9-4366-81C7-84EB6D6C169B}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AE04F058-5A6A-4611-AD8F-2B8A7798BA5F}" name="Table1" displayName="Table1" ref="A1:G24" totalsRowShown="0">
+  <autoFilter ref="A1:G24" xr:uid="{AE04F058-5A6A-4611-AD8F-2B8A7798BA5F}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{582206B5-5641-4C2D-A663-F6AA738E6FB2}" name="Loại"/>
-    <tableColumn id="2" xr3:uid="{06AA52CF-E740-4C10-9531-CF55FBE31A3C}" name="ID"/>
-    <tableColumn id="3" xr3:uid="{E9E89155-6369-4B65-A8B6-49350AFD1271}" name="Trường hợp"/>
-    <tableColumn id="4" xr3:uid="{66B84B2C-B7D5-4C80-9813-ADBE8E8A6812}" name="Đầu vào hoặc thao tác"/>
-    <tableColumn id="5" xr3:uid="{6A4C7699-6628-4A29-9205-08D8E947E027}" name="Kết quả mong đợi"/>
-    <tableColumn id="6" xr3:uid="{924EB3C0-EC05-4614-A080-8FBEE85AD43B}" name="Kết quả thực tế"/>
-    <tableColumn id="7" xr3:uid="{149C1EAF-07CA-4F28-B187-66217DEFBEA8}" name="Trạng thái"/>
+    <tableColumn id="1" xr3:uid="{DE419895-487F-44D6-A5FD-59A7EAAFDA46}" name="Loại"/>
+    <tableColumn id="2" xr3:uid="{567E292B-01BC-4750-B5CC-BF881E3623F9}" name="ID"/>
+    <tableColumn id="3" xr3:uid="{CBC97BE4-D98E-462A-A980-81AAD9684852}" name="Trường hợp"/>
+    <tableColumn id="4" xr3:uid="{CF3C3197-4A59-4935-8546-12791B3FAA74}" name="Đầu vào hoặc thao tác"/>
+    <tableColumn id="5" xr3:uid="{7614F26B-8733-4A6B-AE64-06E8285B6833}" name="Kết quả mong đợi"/>
+    <tableColumn id="6" xr3:uid="{56FF7672-5809-4EE7-87E7-3624E155F064}" name="Kết quả thực tế"/>
+    <tableColumn id="7" xr3:uid="{F2A8BD24-B013-4DBB-8567-176671482D9E}" name="Trạng thái"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -660,528 +690,597 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="43.85546875" customWidth="1"/>
-    <col min="4" max="4" width="88.140625" customWidth="1"/>
-    <col min="5" max="5" width="65.42578125" customWidth="1"/>
-    <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="7" width="13.5703125" customWidth="1"/>
+    <col min="1" max="1" width="9.85546875" customWidth="1"/>
+    <col min="2" max="2" width="20.140625" customWidth="1"/>
+    <col min="3" max="3" width="41.7109375" customWidth="1"/>
+    <col min="4" max="4" width="90.28515625" customWidth="1"/>
+    <col min="5" max="5" width="79.28515625" customWidth="1"/>
+    <col min="6" max="6" width="16.7109375" customWidth="1"/>
+    <col min="7" max="7" width="11.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>26</v>
+        <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>27</v>
+        <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="G1" t="s">
-        <v>29</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="D2" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="E2" t="s">
-        <v>42</v>
+        <v>11</v>
       </c>
       <c r="F2" t="s">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="G2" t="s">
-        <v>44</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="C3" t="s">
-        <v>46</v>
+        <v>15</v>
       </c>
       <c r="D3" t="s">
-        <v>36</v>
+        <v>16</v>
       </c>
       <c r="E3" t="s">
-        <v>45</v>
+        <v>17</v>
       </c>
       <c r="F3" t="s">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="G3" t="s">
-        <v>44</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="C4" t="s">
-        <v>47</v>
+        <v>19</v>
       </c>
       <c r="D4" t="s">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="E4" t="s">
-        <v>48</v>
+        <v>21</v>
       </c>
       <c r="F4" t="s">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="G4" t="s">
-        <v>44</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="C5" t="s">
-        <v>49</v>
+        <v>23</v>
       </c>
       <c r="D5" t="s">
-        <v>51</v>
+        <v>24</v>
       </c>
       <c r="E5" t="s">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="F5" t="s">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="G5" t="s">
-        <v>44</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="B6" t="s">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="C6" t="s">
-        <v>52</v>
+        <v>27</v>
       </c>
       <c r="D6" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="E6" t="s">
-        <v>53</v>
+        <v>29</v>
       </c>
       <c r="F6" t="s">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="G6" t="s">
-        <v>44</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="B7" t="s">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="C7" t="s">
-        <v>54</v>
+        <v>31</v>
       </c>
       <c r="D7" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="E7" t="s">
-        <v>55</v>
+        <v>33</v>
       </c>
       <c r="F7" t="s">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="G7" t="s">
-        <v>44</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>8</v>
+        <v>34</v>
       </c>
       <c r="C8" t="s">
-        <v>56</v>
+        <v>35</v>
       </c>
       <c r="D8" t="s">
-        <v>57</v>
+        <v>36</v>
       </c>
       <c r="E8" t="s">
-        <v>58</v>
+        <v>37</v>
       </c>
       <c r="F8" t="s">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="G8" t="s">
-        <v>44</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>9</v>
+        <v>38</v>
       </c>
       <c r="C9" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="D9" t="s">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="E9" t="s">
-        <v>61</v>
+        <v>41</v>
       </c>
       <c r="F9" t="s">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="G9" t="s">
-        <v>44</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B10" t="s">
-        <v>11</v>
+        <v>89</v>
       </c>
       <c r="C10" t="s">
-        <v>62</v>
+        <v>90</v>
       </c>
       <c r="D10" t="s">
-        <v>35</v>
+        <v>101</v>
       </c>
       <c r="E10" t="s">
-        <v>64</v>
+        <v>91</v>
       </c>
       <c r="F10" t="s">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="G10" t="s">
-        <v>44</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B11" t="s">
-        <v>12</v>
+        <v>92</v>
       </c>
       <c r="C11" t="s">
-        <v>63</v>
+        <v>93</v>
       </c>
       <c r="D11" t="s">
-        <v>40</v>
+        <v>102</v>
       </c>
       <c r="E11" t="s">
-        <v>64</v>
+        <v>94</v>
       </c>
       <c r="F11" t="s">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="G11" t="s">
-        <v>44</v>
+        <v>13</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>42</v>
+      </c>
+      <c r="B12" t="s">
+        <v>43</v>
+      </c>
+      <c r="C12" t="s">
+        <v>44</v>
+      </c>
+      <c r="D12" t="s">
         <v>10</v>
       </c>
-      <c r="B12" t="s">
-        <v>13</v>
-      </c>
-      <c r="C12" t="s">
-        <v>65</v>
-      </c>
-      <c r="D12" t="s">
-        <v>66</v>
-      </c>
       <c r="E12" t="s">
-        <v>67</v>
+        <v>45</v>
       </c>
       <c r="F12" t="s">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="G12" t="s">
-        <v>44</v>
+        <v>13</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="B13" t="s">
-        <v>14</v>
+        <v>46</v>
       </c>
       <c r="C13" t="s">
-        <v>68</v>
+        <v>47</v>
       </c>
       <c r="D13" t="s">
-        <v>69</v>
+        <v>48</v>
       </c>
       <c r="E13" t="s">
-        <v>70</v>
+        <v>45</v>
       </c>
       <c r="F13" t="s">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="G13" t="s">
-        <v>44</v>
+        <v>13</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>15</v>
+        <v>42</v>
       </c>
       <c r="B14" t="s">
-        <v>16</v>
+        <v>49</v>
       </c>
       <c r="C14" t="s">
-        <v>71</v>
+        <v>50</v>
       </c>
       <c r="D14" t="s">
-        <v>72</v>
+        <v>51</v>
       </c>
       <c r="E14" t="s">
-        <v>73</v>
+        <v>52</v>
       </c>
       <c r="F14" t="s">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="G14" t="s">
-        <v>44</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>15</v>
+        <v>42</v>
       </c>
       <c r="B15" t="s">
-        <v>17</v>
+        <v>53</v>
       </c>
       <c r="C15" t="s">
-        <v>74</v>
+        <v>54</v>
       </c>
       <c r="D15" t="s">
-        <v>41</v>
+        <v>55</v>
       </c>
       <c r="E15" t="s">
-        <v>75</v>
+        <v>56</v>
       </c>
       <c r="F15" t="s">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="G15" t="s">
-        <v>44</v>
+        <v>13</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>15</v>
+        <v>57</v>
       </c>
       <c r="B16" t="s">
-        <v>18</v>
+        <v>58</v>
       </c>
       <c r="C16" t="s">
-        <v>76</v>
+        <v>59</v>
       </c>
       <c r="D16" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="E16" t="s">
-        <v>78</v>
+        <v>61</v>
       </c>
       <c r="F16" t="s">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="G16" t="s">
-        <v>44</v>
+        <v>13</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>15</v>
+        <v>57</v>
       </c>
       <c r="B17" t="s">
-        <v>19</v>
+        <v>62</v>
       </c>
       <c r="C17" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="D17" t="s">
-        <v>80</v>
+        <v>64</v>
       </c>
       <c r="E17" t="s">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="F17" t="s">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="G17" t="s">
-        <v>44</v>
+        <v>13</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>15</v>
+        <v>57</v>
       </c>
       <c r="B18" t="s">
-        <v>20</v>
+        <v>66</v>
       </c>
       <c r="C18" t="s">
-        <v>83</v>
+        <v>67</v>
       </c>
       <c r="D18" t="s">
-        <v>81</v>
+        <v>68</v>
       </c>
       <c r="E18" t="s">
-        <v>82</v>
+        <v>69</v>
       </c>
       <c r="F18" t="s">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="G18" t="s">
-        <v>44</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>15</v>
+        <v>57</v>
       </c>
       <c r="B19" t="s">
-        <v>21</v>
+        <v>70</v>
       </c>
       <c r="C19" t="s">
-        <v>84</v>
+        <v>71</v>
       </c>
       <c r="D19" t="s">
-        <v>85</v>
+        <v>72</v>
       </c>
       <c r="E19" t="s">
-        <v>86</v>
+        <v>69</v>
       </c>
       <c r="F19" t="s">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="G19" t="s">
-        <v>44</v>
+        <v>13</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>15</v>
+        <v>57</v>
       </c>
       <c r="B20" t="s">
-        <v>22</v>
+        <v>73</v>
       </c>
       <c r="C20" t="s">
-        <v>91</v>
+        <v>74</v>
       </c>
       <c r="D20" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="E20" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="F20" t="s">
-        <v>89</v>
+        <v>12</v>
       </c>
       <c r="G20" t="s">
-        <v>90</v>
+        <v>13</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>15</v>
+        <v>57</v>
       </c>
       <c r="B21" t="s">
-        <v>23</v>
+        <v>77</v>
       </c>
       <c r="C21" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="D21" t="s">
-        <v>93</v>
+        <v>79</v>
       </c>
       <c r="E21" t="s">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="F21" t="s">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="G21" t="s">
-        <v>44</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>57</v>
+      </c>
+      <c r="B22" t="s">
+        <v>95</v>
+      </c>
+      <c r="C22" t="s">
+        <v>82</v>
+      </c>
+      <c r="D22" t="s">
+        <v>83</v>
+      </c>
+      <c r="E22" t="s">
+        <v>84</v>
+      </c>
+      <c r="F22" t="s">
+        <v>12</v>
+      </c>
+      <c r="G22" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>30</v>
+        <v>57</v>
+      </c>
+      <c r="B23" t="s">
+        <v>81</v>
+      </c>
+      <c r="C23" t="s">
+        <v>96</v>
+      </c>
+      <c r="D23" t="s">
+        <v>103</v>
+      </c>
+      <c r="E23" t="s">
+        <v>97</v>
+      </c>
+      <c r="F23" t="s">
+        <v>12</v>
+      </c>
+      <c r="G23" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>1</v>
+        <v>57</v>
       </c>
       <c r="B24" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>10</v>
-      </c>
-      <c r="B25" t="s">
-        <v>32</v>
+        <v>100</v>
+      </c>
+      <c r="C24" t="s">
+        <v>98</v>
+      </c>
+      <c r="D24" t="s">
+        <v>104</v>
+      </c>
+      <c r="E24" t="s">
+        <v>99</v>
+      </c>
+      <c r="F24" t="s">
+        <v>12</v>
+      </c>
+      <c r="G24" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>15</v>
-      </c>
-      <c r="B26" t="s">
-        <v>33</v>
+        <v>85</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>7</v>
+      </c>
+      <c r="B27" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>42</v>
+      </c>
+      <c r="B28" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>57</v>
+      </c>
+      <c r="B29" t="s">
+        <v>88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>